<commit_message>
docs: 요구사항 완료체크 갱신 — Slice 5(checkin) + PLACE-003 캐싱 반영
- CHECKIN-001~006·008·009·010 + PLACE-003(체크인이 캐싱 upsert 트리거) 완료 처리
- CHECKIN-007(전역 혼밥중 상태바)은 클라 전역상태라 예정 유지
- 체크박스 94개 전부 보존(openpyxl 미사용·zip XML 직접수정), 체크 15→25

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/혼정-기능요구사항-목록.xlsx
+++ b/docs/혼정-기능요구사항-목록.xlsx
@@ -1526,7 +1526,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp24.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp25.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1558,27 +1558,27 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp31.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp32.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp33.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp34.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp35.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp36.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp37.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1586,11 +1586,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp38.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp39.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1598,7 +1598,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp40.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp41.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8689,7 +8689,7 @@
         <v>14</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>16</v>
@@ -8892,7 +8892,7 @@
         <v>14</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>16</v>
@@ -8921,7 +8921,7 @@
         <v>14</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>16</v>
@@ -8950,7 +8950,7 @@
         <v>14</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>16</v>
@@ -8979,7 +8979,7 @@
         <v>14</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>16</v>
@@ -9008,7 +9008,7 @@
         <v>14</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>16</v>
@@ -9037,7 +9037,7 @@
         <v>14</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>16</v>
@@ -9095,7 +9095,7 @@
         <v>14</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>16</v>
@@ -9124,7 +9124,7 @@
         <v>14</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>16</v>
@@ -9153,7 +9153,7 @@
         <v>14</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
docs: 요구사항 완료체크 갱신 — Slice 6(meal) MEAL-001~007
같이먹기 신청·중복/자기차단·opt-out·받은/보낸 목록·수락·거절 7개 완료.
MEAL-008(알림)은 P2 폴링 보류라 제외.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/혼정-기능요구사항-목록.xlsx
+++ b/docs/혼정-기능요구사항-목록.xlsx
@@ -1602,31 +1602,31 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp41.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp42.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp43.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp44.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp45.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp46.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp47.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp48.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9182,7 +9182,7 @@
         <v>14</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>16</v>
@@ -9211,7 +9211,7 @@
         <v>14</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>16</v>
@@ -9240,7 +9240,7 @@
         <v>14</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>16</v>
@@ -9269,7 +9269,7 @@
         <v>14</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>16</v>
@@ -9298,7 +9298,7 @@
         <v>14</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>16</v>
@@ -9327,7 +9327,7 @@
         <v>14</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>16</v>
@@ -9356,7 +9356,7 @@
         <v>14</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>15</v>
+        <v>430</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>16</v>

</xml_diff>